<commit_message>
Replace demo data with Swiss construction project (Überbauung Seefeld)
Complete rework of demo content from German office building to a Swiss
residential/commercial project in Zürich:

Project: "Überbauung Seefeld" — 7-storey mixed-use building
- 48 apartments, ground-floor retail, 68-space underground garage
- CHF 62.8M budget, Minergie-P-ECO certified
- Real Swiss terminology (BKP, SIA, VKF, SIBE, Bausitzung)
- Realistic firms: Implenia, Marti AG, Baumschlager Eberle, etc.

Files (23 total across 8 folders + root):
- Multi-page .docx: Projektbeschrieb, Brandschutzkonzept, Bausitzung
- Multi-page .pdf: 3-page Baubewilligung, 8-page Baufortschrittsbericht
- Professional .xlsx: BKP costs, payment plans, subcontractors, defects
- Construction photos from Unsplash (4 JPGs)
- Markdown project overview

Also fixes document preview scroll cropping in the viewer modal.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-files/01 Planung/Raumprogramm.xlsx
+++ b/demo-files/01 Planung/Raumprogramm.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raumprogramm" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raumprogramm'!$A$1:$F$17</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,8 +28,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,8 +46,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00F2F4F7"/>
+        <bgColor rgb="00F2F4F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -53,10 +60,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00D0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -65,10 +80,10 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,14 +450,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,10 +479,15 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Anzahl Arbeitsplätze</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Zimmer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
@@ -480,20 +501,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Empfang / Lobby</t>
+          <t>Gewerbe A</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>350</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Repräsentativ, doppelte Raumhöhe</t>
+        <v>280</v>
+      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ladenlokal Seefeldstrasse</t>
         </is>
       </c>
     </row>
@@ -505,20 +523,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Konferenzbereich</t>
+          <t>Gewerbe B</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>4 Räume à 20–50 Plätze</t>
+        <v>220</v>
+      </c>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Ladenlokal Seefeldstrasse</t>
         </is>
       </c>
     </row>
@@ -530,20 +545,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Café / Kantine</t>
+          <t>Gewerbe C</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Inkl. Küche</t>
+        <v>180</v>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Gastro / Café mit Terrasse</t>
         </is>
       </c>
     </row>
@@ -555,394 +567,308 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Technik / Nebenräume</t>
+          <t>Eingangsbereich</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Lobby, Briefkästen, Veloabstell</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>1. OG</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fahrradraum / Umkleiden</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>920</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Duschen vorhanden</t>
-        </is>
-      </c>
+          <t>2.5–4.5</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>1. OG</t>
+          <t>2. OG</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Open-Space-Büro</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1100</v>
+        <v>920</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>110</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Flexible Möblierung</t>
-        </is>
-      </c>
+          <t>2.5–4.5</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>1. OG</t>
+          <t>3. OG</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Besprechungsräume</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>920</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>6 Räume</t>
-        </is>
-      </c>
+          <t>2.5–4.5</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>1. OG</t>
+          <t>4. OG</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Teeküche / Sozialräume</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+        <v>880</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>3.5–5.5</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Grösserer Grundriss</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2. OG</t>
+          <t>5. OG</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Open-Space-Büro</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1100</v>
+        <v>880</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>110</v>
+        <v>6</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Flexible Möblierung</t>
-        </is>
-      </c>
+          <t>3.5–5.5</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2. OG</t>
+          <t>6. OG</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Besprechungsräume</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>760</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>6 Räume</t>
-        </is>
-      </c>
+          <t>4.5–5.5</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2. OG</t>
+          <t>Attika</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Teeküche / Sozialräume</t>
+          <t>Wohnungen</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+        <v>520</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>4.5–5.5</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Mit Dachterrassen</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3. OG</t>
+          <t>Attika</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Open-Space-Büro</t>
+          <t>Gemeinschaftsterrasse</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+        <v>180</v>
+      </c>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Zugänglich für alle Bewohner</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3. OG</t>
+          <t>1. UG</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Besprechungsräume</t>
+          <t>Tiefgarage</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>4 Räume</t>
+        <v>2400</v>
+      </c>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>68 PP, Velokeller, Waschküche</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3. OG</t>
+          <t>2. UG</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Serverraum</t>
+          <t>Technik / Keller</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Klimatisiert</t>
+        <v>1800</v>
+      </c>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>HLKS-Zentrale, Kellerabteile</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4. OG</t>
+          <t>Dach</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Open-Space-Büro</t>
+          <t>PV-Anlage</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+        <v>620</v>
+      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>180 kWp</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>4. OG</t>
+          <t>Dach</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Besprechungsräume</t>
+          <t>Biodiversitätsdach</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>4 Räume</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>5. OG</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Geschäftsleitung</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>600</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Einzelbüros + Assistenz</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>5. OG</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Executive Lounge</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Inkl. Dachterrasse</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>UG1</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Tiefgarage</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>2100</v>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>120 Stellplätze</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>UG2</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Tiefgarage + Technik</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2100</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>60 Stellplätze + Haustechnik</t>
+        <v>330</v>
+      </c>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Extensivbegrünung</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>